<commit_message>
Roadmap Excel: zeus 2.0.x sürüm satırı ve geriye uyumsuzluk ifadeleri güncellendi
- BOM/sürüm kolonları 1.1.x → 2.0.x, tarih Haz 2026
- spring-ai-bom satırı 2.0.x (Boot 4 gerektirir) olarak netleştirildi
- "kırıcı sürüm" ifadeleri "geriye uyumsuz (breaking) — pom değişikliği zorunlu" şeklinde açıldı
</commit_message>
<xml_diff>
--- a/framework-upgrade-roadmap.xlsx
+++ b/framework-upgrade-roadmap.xlsx
@@ -657,7 +657,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Zeus Framework 1.x → 2.0.0 (kırıcı platform sürümü) + tüketici uygulamaların geçişi</t>
+          <t>Zeus Framework 1.x → 2.0.0 — geriye uyumsuz (breaking) platform sürümü: uygulamalarda pom değişikliği zorunlu — + tüketici uygulamaların geçişi</t>
         </is>
       </c>
       <c r="C4" s="5" t="n"/>
@@ -1304,12 +1304,12 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>1.1.x (BOM)</t>
+          <t>2.0.x (BOM)</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>PLANLANAN: zeus-ai-mcp modülü — kurumsal uygulamaların servislerini MCP (Model Context Protocol) üzerinden AI ajanlarına tool olarak açması + MCP client tüketimi. Spring AI'ın resmi MCP server/client starter'ları Boot 4 satırıyla hizalanınca BOM'a spring-ai-bom eklenecek.</t>
+          <t>PLANLANAN: zeus-ai-mcp modülü — kurumsal uygulamaların servislerini MCP (Model Context Protocol) üzerinden AI ajanlarına tool olarak açması + MCP client tüketimi. Spring AI 2.0 (Haz 2026 GA) Boot 4.0 GEREKTİRİR — stack'imizle birebir hizalı; 1.x satırı Boot 3 içindir ve kullanılamaz. BOM'a spring-ai-bom 2.0.x eklenecek.</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -1747,12 +1747,12 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>1.1.x</t>
+          <t>2.0.x</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>2025–2026</t>
+          <t>Haz 2026</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>zeus-ai-mcp için; MCP starter'ları hızlı evriliyor — BOM pinleme şart</t>
+          <t>zeus-ai-mcp için; 2.0 Boot 4 gerektirir (1.x = Boot 3 satırı). MCP starter'ları hızlı evriliyor — BOM pinleme şart</t>
         </is>
       </c>
     </row>
@@ -1923,7 +1923,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Analiz &amp; sürüm kararları (Java 25 / Boot 4.0.7 / WF41 seçimi, kırıcılık analizi, semver kararı)</t>
+          <t>Analiz &amp; sürüm kararları: hedef sürüm seçimi (Java 25 / Boot 4.0.7 / WF41) + Boot 3→4'te uygulamaları etkileyecek değişikliklerin çıkarılması (starter adları, property'ler, springdoc) + zeus sürüm numarası kararı (pom değişikliği zorunlu → major, 2.0.0)</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -1954,7 +1954,7 @@
       <c r="J5" s="8" t="inlineStr"/>
       <c r="K5" s="8" t="inlineStr">
         <is>
-          <t>2.0.0 kırıcı sürüm kararı</t>
+          <t>Sonuç: geriye uyumsuz → zeus 2.0.0</t>
         </is>
       </c>
     </row>
@@ -3077,7 +3077,7 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>spring-ai-bom (Boot 4 uyumlu satır) · zeus-base</t>
+          <t>spring-ai-bom 2.0.x (Boot 4 gerektirir) · zeus-base</t>
         </is>
       </c>
       <c r="F5" s="19" t="inlineStr">

</xml_diff>